<commit_message>
docs: complete issue 027 security assessment
</commit_message>
<xml_diff>
--- a/docs/OffSec_Lab_v0.1_WBS.xlsx
+++ b/docs/OffSec_Lab_v0.1_WBS.xlsx
@@ -2372,7 +2372,7 @@
                   <c:v>Phase 9: Testing</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Phase 10: Security Assessment</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>Phase 11: Documentation</c:v>
@@ -3087,7 +3087,7 @@
       </c>
       <c r="B5" s="9">
         <f>COUNTIF(WBS!L4:L79,"Done")</f>
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="8" t="s">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="E5" s="9">
         <f>COUNTIF('Codex Issues'!I4:I32,"Done")</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="B8" s="10">
         <f>AVERAGE(WBS!M4:M79)</f>
-        <v>0.84868421052631582</v>
+        <v>0.9407894736842105</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="s">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="E8" s="9">
         <f>COUNTIF(Milestones!F4:F11,"Done")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F8" s="7"/>
       <c r="G8" s="7"/>
@@ -3313,8 +3313,8 @@
         <v>653</v>
       </c>
       <c r="G15" s="7" t="str">
-        <f>IF(Milestones!F9="Done",'Codex Issues'!D30,'Codex Issues'!D26)</f>
-        <v>Phase 10</v>
+        <f>IF(Milestones!F10="Done",'Codex Issues'!D31,'Codex Issues'!D30)</f>
+        <v>Phase 11</v>
       </c>
       <c r="H15" s="7"/>
     </row>
@@ -3339,8 +3339,8 @@
         <v>654</v>
       </c>
       <c r="G16" s="7" t="str">
-        <f>IF(Milestones!F9="Done",'Codex Issues'!A30,'Codex Issues'!A26)</f>
-        <v>ISSUE-027</v>
+        <f>IF(Milestones!F10="Done",'Codex Issues'!A31,'Codex Issues'!A30)</f>
+        <v>ISSUE-028</v>
       </c>
       <c r="H16" s="7"/>
     </row>
@@ -3469,11 +3469,11 @@
       </c>
       <c r="C22" s="7">
         <f>COUNTIFS(WBS!B4:B79,A22,WBS!L4:L79,"Done")</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D22" s="13">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="14" t="s">
@@ -6088,11 +6088,11 @@
       <c r="J67" s="4"/>
       <c r="K67" s="4"/>
       <c r="L67" s="4" t="s">
-        <v>650</v>
+        <v>4</v>
       </c>
       <c r="M67" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68" spans="1:13" ht="28.5">
@@ -6126,11 +6126,11 @@
       <c r="J68" s="4"/>
       <c r="K68" s="4"/>
       <c r="L68" s="4" t="s">
-        <v>650</v>
+        <v>4</v>
       </c>
       <c r="M68" s="5">
         <f t="shared" ref="M68:M79" si="2">IF(L68="Done",1,IF(L68="In Progress",0.5,IF(L68="Blocked",0.25,0)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:13" ht="28.5">
@@ -6164,11 +6164,11 @@
       <c r="J69" s="4"/>
       <c r="K69" s="4"/>
       <c r="L69" s="4" t="s">
-        <v>650</v>
+        <v>4</v>
       </c>
       <c r="M69" s="5">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:13" ht="28.5">
@@ -6202,11 +6202,11 @@
       <c r="J70" s="4"/>
       <c r="K70" s="4"/>
       <c r="L70" s="4" t="s">
-        <v>650</v>
+        <v>4</v>
       </c>
       <c r="M70" s="5">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71" spans="1:13" ht="28.5">
@@ -6240,11 +6240,11 @@
       <c r="J71" s="4"/>
       <c r="K71" s="4"/>
       <c r="L71" s="4" t="s">
-        <v>650</v>
+        <v>4</v>
       </c>
       <c r="M71" s="5">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72" spans="1:13" ht="28.5">
@@ -6278,11 +6278,11 @@
       <c r="J72" s="4"/>
       <c r="K72" s="4"/>
       <c r="L72" s="4" t="s">
-        <v>650</v>
+        <v>4</v>
       </c>
       <c r="M72" s="5">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" spans="1:13" ht="28.5">
@@ -6316,11 +6316,11 @@
       <c r="J73" s="4"/>
       <c r="K73" s="4"/>
       <c r="L73" s="4" t="s">
-        <v>650</v>
+        <v>4</v>
       </c>
       <c r="M73" s="5">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74" spans="1:13" ht="42.75">
@@ -7580,11 +7580,11 @@
         <v>594</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>650</v>
+        <v>4</v>
       </c>
       <c r="J30" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:10">
@@ -7924,7 +7924,7 @@
         <v>643</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>650</v>
+        <v>4</v>
       </c>
       <c r="G10" s="4"/>
     </row>

</xml_diff>

<commit_message>
docs: finalize v0.1 documentation for ISSUE-028
</commit_message>
<xml_diff>
--- a/docs/OffSec_Lab_v0.1_WBS.xlsx
+++ b/docs/OffSec_Lab_v0.1_WBS.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R67e73c3fd2fe4be4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="Rd88025a0c79246ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Issues" sheetId="3" r:id="Rfd803fd11c23405c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="Rd86ad0d412ac4b44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="5" r:id="Rd99f041efb884d15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf4022f6e0afd4f15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="Rabc233156c074a73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codex Issues" sheetId="3" r:id="R7f253e456c874031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="R7dee5f625bba4120"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master" sheetId="5" r:id="Rb62f7a4eedac4a4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1379,55 +1379,55 @@
     <x:t xml:space="preserve">Security Assessment結果が反映されている</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">11.4</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Test Report</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">実施テストと結果を記録する。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Test report</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">主要Testの結果とEvidenceが記録されている</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">11.5</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Development Log</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">判断・問題・解決・学習を記録する。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Development log</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">ポートフォリオで開発プロセスを説明できる</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">12.1</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">MVP Acceptance Review</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">v0.1受入基準を全件確認し、MVP完成判定を行う。</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">11.1,11.2,11.3,11.4</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">MVP acceptance record</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">全必須Acceptance Criteriaを満たす</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">Not Started</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">11.4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Test Report</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">実施テストと結果を記録する。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Test report</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">主要Testの結果とEvidenceが記録されている</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">11.5</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Development Log</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">判断・問題・解決・学習を記録する。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Development log</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ポートフォリオで開発プロセスを説明できる</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">12.1</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">MVP Acceptance Review</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">v0.1受入基準を全件確認し、MVP完成判定を行う。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">11.1,11.2,11.3,11.4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">MVP acceptance record</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">全必須Acceptance Criteriaを満たす</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">OffSec Lab v0.1 — Codex Issue Backlog</x:t>
@@ -2687,7 +2687,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfef5d2c7e53f4a6a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R58de14d47bcc4b45"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3000,7 +3000,7 @@
       </x:c>
       <x:c r="B5" s="9" t="n">
         <x:f>COUNTIF(WBS!L4:L79,"Done")</x:f>
-        <x:v>71</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C5" s="7"/>
       <x:c r="D5" s="8" t="s">
@@ -3008,7 +3008,7 @@
       </x:c>
       <x:c r="E5" s="9" t="n">
         <x:f>COUNTIF('Codex Issues'!I4:I32,"Done")</x:f>
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="F5" s="7"/>
       <x:c r="G5" s="7"/>
@@ -3020,7 +3020,7 @@
       </x:c>
       <x:c r="B6" s="9" t="n">
         <x:f>COUNTIF(WBS!L4:L79,"In Progress")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="7"/>
       <x:c r="D6" s="8" t="s">
@@ -3060,7 +3060,7 @@
       </x:c>
       <x:c r="B8" s="10" t="n">
         <x:f>AVERAGE(WBS!M4:M79)</x:f>
-        <x:v>0.9473684210526315</x:v>
+        <x:v>0.9868421052631579</x:v>
       </x:c>
       <x:c r="C8" s="7"/>
       <x:c r="D8" s="8" t="s">
@@ -3226,8 +3226,8 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="G15" s="7" t="str">
-        <x:f>IF(Milestones!F10="Done",'Codex Issues'!D31,'Codex Issues'!D30)</x:f>
-        <x:v>Phase 11</x:v>
+        <x:f>IF(COUNTIF('Codex Issues'!I4:I32,"In Progress")&gt;0,INDEX('Codex Issues'!D4:D32,MATCH("In Progress",'Codex Issues'!I4:I32,0)),IF(COUNTIF('Codex Issues'!I4:I32,"Blocked")&gt;0,INDEX('Codex Issues'!D4:D32,MATCH("Blocked",'Codex Issues'!I4:I32,0)),IF(COUNTIF('Codex Issues'!I4:I32,"Not Started")&gt;0,INDEX('Codex Issues'!D4:D32,MATCH("Not Started",'Codex Issues'!I4:I32,0)),"Complete")))</x:f>
+        <x:v>Phase 12</x:v>
       </x:c>
       <x:c r="H15" s="7"/>
     </x:row>
@@ -3252,8 +3252,8 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="G16" s="7" t="str">
-        <x:f>IF(Milestones!F10="Done",'Codex Issues'!A31,'Codex Issues'!A30)</x:f>
-        <x:v>ISSUE-028</x:v>
+        <x:f>IF(COUNTIF('Codex Issues'!I4:I32,"In Progress")&gt;0,INDEX('Codex Issues'!A4:A32,MATCH("In Progress",'Codex Issues'!I4:I32,0)),IF(COUNTIF('Codex Issues'!I4:I32,"Blocked")&gt;0,INDEX('Codex Issues'!A4:A32,MATCH("Blocked",'Codex Issues'!I4:I32,0)),IF(COUNTIF('Codex Issues'!I4:I32,"Not Started")&gt;0,INDEX('Codex Issues'!A4:A32,MATCH("Not Started",'Codex Issues'!I4:I32,0)),"None")))</x:f>
+        <x:v>ISSUE-029</x:v>
       </x:c>
       <x:c r="H16" s="7"/>
     </x:row>
@@ -3405,11 +3405,11 @@
       </x:c>
       <x:c r="C23" s="7" t="n">
         <x:f>COUNTIFS(WBS!B4:B79,A23,WBS!L4:L79,"Done")</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D23" s="13">
-        <x:f t="shared" si="0"/>
-        <x:v>0.2</x:v>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D23" s="13" t="n">
+        <x:f t="shared" si="0">IF(B23=0,0,C23/B23)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E23" s="7"/>
       <x:c r="F23" s="15" t="s">
@@ -3480,7 +3480,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79d10d8c5c204207"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cc3484dc47547fc"/>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
@@ -6265,12 +6265,12 @@
       </x:c>
       <x:c r="J74" s="4"/>
       <x:c r="K74" s="4"/>
-      <x:c r="L74" s="4" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="M74" s="5">
-        <x:f t="shared" si="2"/>
-        <x:v>0.5</x:v>
+      <x:c r="L74" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="M74" s="5" t="n">
+        <x:f t="shared" si="2">IF(L74="Done",1,IF(L74="In Progress",0.5,IF(L74="Blocked",0.25,0)))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="28.5">
@@ -6303,12 +6303,12 @@
       </x:c>
       <x:c r="J75" s="4"/>
       <x:c r="K75" s="4"/>
-      <x:c r="L75" s="4" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="M75" s="5">
-        <x:f t="shared" si="2"/>
-        <x:v>0.5</x:v>
+      <x:c r="L75" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="M75" s="5" t="n">
+        <x:f t="shared" si="2">IF(L75="Done",1,IF(L75="In Progress",0.5,IF(L75="Blocked",0.25,0)))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="15">
@@ -6341,26 +6341,26 @@
       </x:c>
       <x:c r="J76" s="4"/>
       <x:c r="K76" s="4"/>
-      <x:c r="L76" s="4" t="s">
-        <x:v>455</x:v>
-      </x:c>
-      <x:c r="M76" s="5">
-        <x:f t="shared" si="2"/>
-        <x:v>0</x:v>
+      <x:c r="L76" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="M76" s="5" t="n">
+        <x:f t="shared" si="2">IF(L76="Done",1,IF(L76="In Progress",0.5,IF(L76="Blocked",0.25,0)))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="15">
       <x:c r="A77" s="4" t="s">
-        <x:v>456</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="B77" s="4" t="s">
         <x:v>40</x:v>
       </x:c>
       <x:c r="C77" s="4" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="D77" s="4" t="s">
         <x:v>457</x:v>
-      </x:c>
-      <x:c r="D77" s="4" t="s">
-        <x:v>458</x:v>
       </x:c>
       <x:c r="E77" s="4" t="s">
         <x:v>394</x:v>
@@ -6372,10 +6372,10 @@
         <x:v>398</x:v>
       </x:c>
       <x:c r="H77" s="4" t="s">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="I77" s="4" t="s">
         <x:v>459</x:v>
-      </x:c>
-      <x:c r="I77" s="4" t="s">
-        <x:v>460</x:v>
       </x:c>
       <x:c r="J77" s="4"/>
       <x:c r="K77" s="4"/>
@@ -6389,16 +6389,16 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="4" t="s">
-        <x:v>461</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="B78" s="4" t="s">
         <x:v>40</x:v>
       </x:c>
       <x:c r="C78" s="4" t="s">
+        <x:v>461</x:v>
+      </x:c>
+      <x:c r="D78" s="4" t="s">
         <x:v>462</x:v>
-      </x:c>
-      <x:c r="D78" s="4" t="s">
-        <x:v>463</x:v>
       </x:c>
       <x:c r="E78" s="4" t="s">
         <x:v>76</x:v>
@@ -6410,33 +6410,33 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="H78" s="4" t="s">
+        <x:v>463</x:v>
+      </x:c>
+      <x:c r="I78" s="4" t="s">
         <x:v>464</x:v>
-      </x:c>
-      <x:c r="I78" s="4" t="s">
-        <x:v>465</x:v>
       </x:c>
       <x:c r="J78" s="4"/>
       <x:c r="K78" s="4"/>
-      <x:c r="L78" s="4" t="s">
-        <x:v>455</x:v>
-      </x:c>
-      <x:c r="M78" s="5">
-        <x:f t="shared" si="2"/>
-        <x:v>0</x:v>
+      <x:c r="L78" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="M78" s="5" t="n">
+        <x:f t="shared" si="2">IF(L78="Done",1,IF(L78="In Progress",0.5,IF(L78="Blocked",0.25,0)))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="28.5">
       <x:c r="A79" s="4" t="s">
-        <x:v>466</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="B79" s="4" t="s">
         <x:v>42</x:v>
       </x:c>
       <x:c r="C79" s="4" t="s">
+        <x:v>466</x:v>
+      </x:c>
+      <x:c r="D79" s="4" t="s">
         <x:v>467</x:v>
-      </x:c>
-      <x:c r="D79" s="4" t="s">
-        <x:v>468</x:v>
       </x:c>
       <x:c r="E79" s="4" t="s">
         <x:v>76</x:v>
@@ -6445,18 +6445,18 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="G79" s="4" t="s">
+        <x:v>468</x:v>
+      </x:c>
+      <x:c r="H79" s="4" t="s">
         <x:v>469</x:v>
       </x:c>
-      <x:c r="H79" s="4" t="s">
+      <x:c r="I79" s="4" t="s">
         <x:v>470</x:v>
-      </x:c>
-      <x:c r="I79" s="4" t="s">
-        <x:v>471</x:v>
       </x:c>
       <x:c r="J79" s="4"/>
       <x:c r="K79" s="4"/>
       <x:c r="L79" s="4" t="s">
-        <x:v>455</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="M79" s="5">
         <x:f t="shared" si="2"/>
@@ -6524,7 +6524,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3feb4763f474aaf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6db0297fef6430e"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -7523,12 +7523,12 @@
       <x:c r="H31" s="4" t="s">
         <x:v>605</x:v>
       </x:c>
-      <x:c r="I31" s="4" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="J31" s="5">
-        <x:f t="shared" si="0"/>
-        <x:v>0.5</x:v>
+      <x:c r="I31" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="J31" s="5" t="n">
+        <x:f t="shared" si="0">IF(I31="Done",1,IF(I31="In Progress",0.5,IF(I31="Blocked",0.25,0)))</x:f>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -7536,7 +7536,7 @@
         <x:v>606</x:v>
       </x:c>
       <x:c r="B32" s="4" t="s">
-        <x:v>467</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="C32" s="4" t="s">
         <x:v>607</x:v>
@@ -7556,8 +7556,8 @@
       <x:c r="H32" s="4" t="s">
         <x:v>609</x:v>
       </x:c>
-      <x:c r="I32" s="4" t="s">
-        <x:v>455</x:v>
+      <x:c r="I32" s="4" t="str">
+        <x:v>Not Started</x:v>
       </x:c>
       <x:c r="J32" s="5">
         <x:f t="shared" si="0"/>
@@ -7617,7 +7617,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f4d8288c3db4d54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d9d0688cda345d6"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -7855,7 +7855,7 @@
         <x:v>656</x:v>
       </x:c>
       <x:c r="F11" s="4" t="s">
-        <x:v>455</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="G11" s="4"/>
     </x:row>
@@ -7881,7 +7881,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1739a0e8da3c4bbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12b488a46ed448f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7910,7 +7910,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="s">
-        <x:v>455</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="B2" t="s">
         <x:v>19</x:v>

</xml_diff>

<commit_message>
docs: record OffSec Lab v0.1 MVP acceptance
</commit_message>
<xml_diff>
--- a/docs/OffSec_Lab_v0.1_WBS.xlsx
+++ b/docs/OffSec_Lab_v0.1_WBS.xlsx
@@ -3000,7 +3000,7 @@
       </x:c>
       <x:c r="B5" s="9" t="n">
         <x:f>COUNTIF(WBS!L4:L79,"Done")</x:f>
-        <x:v>75</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C5" s="7"/>
       <x:c r="D5" s="8" t="s">
@@ -3008,7 +3008,7 @@
       </x:c>
       <x:c r="E5" s="9" t="n">
         <x:f>COUNTIF('Codex Issues'!I4:I32,"Done")</x:f>
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F5" s="7"/>
       <x:c r="G5" s="7"/>
@@ -3060,7 +3060,7 @@
       </x:c>
       <x:c r="B8" s="10" t="n">
         <x:f>AVERAGE(WBS!M4:M79)</x:f>
-        <x:v>0.9868421052631579</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C8" s="7"/>
       <x:c r="D8" s="8" t="s">
@@ -3068,7 +3068,7 @@
       </x:c>
       <x:c r="E8" s="9" t="n">
         <x:f>COUNTIF(Milestones!F4:F11,"Done")</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F8" s="7"/>
       <x:c r="G8" s="7"/>
@@ -3227,7 +3227,7 @@
       </x:c>
       <x:c r="G15" s="7" t="str">
         <x:f>IF(COUNTIF('Codex Issues'!I4:I32,"In Progress")&gt;0,INDEX('Codex Issues'!D4:D32,MATCH("In Progress",'Codex Issues'!I4:I32,0)),IF(COUNTIF('Codex Issues'!I4:I32,"Blocked")&gt;0,INDEX('Codex Issues'!D4:D32,MATCH("Blocked",'Codex Issues'!I4:I32,0)),IF(COUNTIF('Codex Issues'!I4:I32,"Not Started")&gt;0,INDEX('Codex Issues'!D4:D32,MATCH("Not Started",'Codex Issues'!I4:I32,0)),"Complete")))</x:f>
-        <x:v>Phase 12</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="H15" s="7"/>
     </x:row>
@@ -3253,7 +3253,7 @@
       </x:c>
       <x:c r="G16" s="7" t="str">
         <x:f>IF(COUNTIF('Codex Issues'!I4:I32,"In Progress")&gt;0,INDEX('Codex Issues'!A4:A32,MATCH("In Progress",'Codex Issues'!I4:I32,0)),IF(COUNTIF('Codex Issues'!I4:I32,"Blocked")&gt;0,INDEX('Codex Issues'!A4:A32,MATCH("Blocked",'Codex Issues'!I4:I32,0)),IF(COUNTIF('Codex Issues'!I4:I32,"Not Started")&gt;0,INDEX('Codex Issues'!A4:A32,MATCH("Not Started",'Codex Issues'!I4:I32,0)),"None")))</x:f>
-        <x:v>ISSUE-029</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="H16" s="7"/>
     </x:row>
@@ -3428,11 +3428,11 @@
       </x:c>
       <x:c r="C24" s="7" t="n">
         <x:f>COUNTIFS(WBS!B4:B79,A24,WBS!L4:L79,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D24" s="13">
         <x:f t="shared" si="0"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E24" s="7"/>
       <x:c r="F24" s="7"/>
@@ -6425,7 +6425,7 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="79" ht="28.5">
+    <x:row r="79" ht="42.75" customHeight="1">
       <x:c r="A79" s="4" t="s">
         <x:v>465</x:v>
       </x:c>
@@ -6447,20 +6447,20 @@
       <x:c r="G79" s="4" t="s">
         <x:v>468</x:v>
       </x:c>
-      <x:c r="H79" s="4" t="s">
-        <x:v>469</x:v>
+      <x:c r="H79" s="4" t="str">
+        <x:v>ISSUE-029: all categories PASS; Product Owner approval recorded</x:v>
       </x:c>
       <x:c r="I79" s="4" t="s">
         <x:v>470</x:v>
       </x:c>
       <x:c r="J79" s="4"/>
       <x:c r="K79" s="4"/>
-      <x:c r="L79" s="4" t="s">
-        <x:v>471</x:v>
+      <x:c r="L79" s="4" t="str">
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="M79" s="5">
         <x:f t="shared" si="2"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7557,11 +7557,11 @@
         <x:v>609</x:v>
       </x:c>
       <x:c r="I32" s="4" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="J32" s="5">
         <x:f t="shared" si="0"/>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7838,7 +7838,7 @@
       </x:c>
       <x:c r="G10" s="4"/>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="42.75" customHeight="1">
       <x:c r="A11" s="4" t="s">
         <x:v>652</x:v>
       </x:c>
@@ -7854,10 +7854,12 @@
       <x:c r="E11" s="4" t="s">
         <x:v>656</x:v>
       </x:c>
-      <x:c r="F11" s="4" t="s">
-        <x:v>471</x:v>
-      </x:c>
-      <x:c r="G11" s="4"/>
+      <x:c r="F11" s="4" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G11" s="4" t="str">
+        <x:v>MVP review passed; Product Owner approval recorded; OffSec Lab v0.1 accepted.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>